<commit_message>
fix(taipei-dome): 版本 2 依 code review 修正同列穿越與頁面標示
- 同一列依格位順序抵達：離走道近的人在座位多等，不再穿過同列已站好的人
- check.py 改為同列也計入、0.05 秒取樣：修正前 143 人穿越（全為同列），修正後 0
- 排程每輪各鏈各修一列，迭代 24 → 8 輪；first_in_zone 改寫清楚、移除未用程式
- 白衣 2–9 的「樓梯三路第幾路」改為實際走的路；B2 藍衣區標記移到區頭；集結點標記改用先進場大隊的顏色
- 說明統一為「鏈 A 靠看台」；移除「6藍」等版本 1 用語，個人卡片改為「B2/B1 集結」「集結區 1」
- 版本 1、2 頁首互連連結加上樣式（深色可讀、手機好點）
- 全長 4 分 33 秒 → 5 分 4 秒（同列等候的代價），excel 依新時間重產

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M2sMindg5j1TuA3wvLat6x
</commit_message>
<xml_diff>
--- a/design-explorations/taipei-dome/flow/entry-animation-v2/休息區座位_藍衣B2集結版_2026-10-18.xlsx
+++ b/design-explorations/taipei-dome/flow/entry-animation-v2/休息區座位_藍衣B2集結版_2026-10-18.xlsx
@@ -21279,7 +21279,7 @@
       </c>
       <c r="G5" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">大隊 1(1:54)</t>
+          <t xml:space="preserve">大隊 1(2:10)</t>
         </is>
       </c>
     </row>
@@ -21314,7 +21314,7 @@
       </c>
       <c r="G6" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">大隊 2(2:11)、大隊 3(2:27)</t>
+          <t xml:space="preserve">大隊 2(2:27)、大隊 3(2:42)</t>
         </is>
       </c>
     </row>
@@ -21349,7 +21349,7 @@
       </c>
       <c r="G7" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">大隊 4(2:41)、大隊 5(2:57)</t>
+          <t xml:space="preserve">大隊 4(3:00)、大隊 5(3:15)</t>
         </is>
       </c>
     </row>
@@ -21384,7 +21384,7 @@
       </c>
       <c r="G8" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">大隊 6(3:14)、大隊 7(3:47)</t>
+          <t xml:space="preserve">大隊 6(3:40)、大隊 7(4:17)</t>
         </is>
       </c>
     </row>
@@ -21419,7 +21419,7 @@
       </c>
       <c r="G9" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">大隊 8(4:03)、大隊 9(4:17)</t>
+          <t xml:space="preserve">大隊 8(4:33)、大隊 9(4:47)</t>
         </is>
       </c>
     </row>
@@ -21454,7 +21454,7 @@
       </c>
       <c r="G10" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">大隊 2(2:11)</t>
+          <t xml:space="preserve">大隊 2(2:26)</t>
         </is>
       </c>
     </row>
@@ -21489,7 +21489,7 @@
       </c>
       <c r="G11" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">大隊 3(2:26)</t>
+          <t xml:space="preserve">大隊 3(2:42)</t>
         </is>
       </c>
     </row>
@@ -21524,7 +21524,7 @@
       </c>
       <c r="G12" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">大隊 4(2:41)、大隊 5(2:56)</t>
+          <t xml:space="preserve">大隊 4(3:00)、大隊 5(3:15)</t>
         </is>
       </c>
     </row>
@@ -21559,7 +21559,7 @@
       </c>
       <c r="G13" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">大隊 6(3:13)、大隊 7(3:46)</t>
+          <t xml:space="preserve">大隊 6(3:39)、大隊 7(4:17)</t>
         </is>
       </c>
     </row>
@@ -21594,7 +21594,7 @@
       </c>
       <c r="G14" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">大隊 8(4:02)、大隊 9(4:16)</t>
+          <t xml:space="preserve">大隊 8(4:33)、大隊 9(4:47)</t>
         </is>
       </c>
     </row>
@@ -21718,17 +21718,17 @@
       </c>
       <c r="K18" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:30</t>
+          <t xml:space="preserve">1:43</t>
         </is>
       </c>
       <c r="L18" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:48</t>
+          <t xml:space="preserve">2:03</t>
         </is>
       </c>
       <c r="M18" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:54</t>
+          <t xml:space="preserve">2:10</t>
         </is>
       </c>
     </row>
@@ -21777,17 +21777,17 @@
       </c>
       <c r="K19" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:39</t>
+          <t xml:space="preserve">1:54</t>
         </is>
       </c>
       <c r="L19" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:01</t>
+          <t xml:space="preserve">2:17</t>
         </is>
       </c>
       <c r="M19" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:55</t>
+          <t xml:space="preserve">2:10</t>
         </is>
       </c>
     </row>
@@ -21836,17 +21836,17 @@
       </c>
       <c r="K20" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:40</t>
+          <t xml:space="preserve">1:55</t>
         </is>
       </c>
       <c r="L20" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:02</t>
+          <t xml:space="preserve">2:18</t>
         </is>
       </c>
       <c r="M20" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:55</t>
+          <t xml:space="preserve">2:10</t>
         </is>
       </c>
     </row>
@@ -21895,17 +21895,17 @@
       </c>
       <c r="K21" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:30</t>
+          <t xml:space="preserve">1:43</t>
         </is>
       </c>
       <c r="L21" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:49</t>
+          <t xml:space="preserve">2:04</t>
         </is>
       </c>
       <c r="M21" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:55</t>
+          <t xml:space="preserve">2:10</t>
         </is>
       </c>
     </row>
@@ -21954,17 +21954,17 @@
       </c>
       <c r="K22" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:32</t>
+          <t xml:space="preserve">1:45</t>
         </is>
       </c>
       <c r="L22" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:50</t>
+          <t xml:space="preserve">2:05</t>
         </is>
       </c>
       <c r="M22" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:55</t>
+          <t xml:space="preserve">2:11</t>
         </is>
       </c>
     </row>
@@ -22013,17 +22013,17 @@
       </c>
       <c r="K23" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:43</t>
+          <t xml:space="preserve">1:58</t>
         </is>
       </c>
       <c r="L23" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:01</t>
+          <t xml:space="preserve">2:17</t>
         </is>
       </c>
       <c r="M23" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:55</t>
+          <t xml:space="preserve">2:11</t>
         </is>
       </c>
     </row>
@@ -22072,17 +22072,17 @@
       </c>
       <c r="K24" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:50</t>
+          <t xml:space="preserve">2:06</t>
         </is>
       </c>
       <c r="L24" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:11</t>
+          <t xml:space="preserve">2:28</t>
         </is>
       </c>
       <c r="M24" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:11</t>
+          <t xml:space="preserve">2:26</t>
         </is>
       </c>
     </row>
@@ -22131,17 +22131,17 @@
       </c>
       <c r="K25" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:50</t>
+          <t xml:space="preserve">2:06</t>
         </is>
       </c>
       <c r="L25" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:11</t>
+          <t xml:space="preserve">2:28</t>
         </is>
       </c>
       <c r="M25" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:11</t>
+          <t xml:space="preserve">2:26</t>
         </is>
       </c>
     </row>
@@ -22190,17 +22190,17 @@
       </c>
       <c r="K26" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:55</t>
+          <t xml:space="preserve">2:11</t>
         </is>
       </c>
       <c r="L26" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:12</t>
+          <t xml:space="preserve">2:29</t>
         </is>
       </c>
       <c r="M26" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:11</t>
+          <t xml:space="preserve">2:27</t>
         </is>
       </c>
     </row>
@@ -22249,17 +22249,17 @@
       </c>
       <c r="K27" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:11</t>
+          <t xml:space="preserve">1:21</t>
         </is>
       </c>
       <c r="L27" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:30</t>
+          <t xml:space="preserve">1:41</t>
         </is>
       </c>
       <c r="M27" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:11</t>
+          <t xml:space="preserve">2:27</t>
         </is>
       </c>
     </row>
@@ -22308,17 +22308,17 @@
       </c>
       <c r="K28" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:09</t>
+          <t xml:space="preserve">1:19</t>
         </is>
       </c>
       <c r="L28" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:29</t>
+          <t xml:space="preserve">1:41</t>
         </is>
       </c>
       <c r="M28" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:12</t>
+          <t xml:space="preserve">2:27</t>
         </is>
       </c>
     </row>
@@ -22367,17 +22367,17 @@
       </c>
       <c r="K29" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:19</t>
+          <t xml:space="preserve">1:30</t>
         </is>
       </c>
       <c r="L29" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:40</t>
+          <t xml:space="preserve">1:53</t>
         </is>
       </c>
       <c r="M29" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:12</t>
+          <t xml:space="preserve">2:27</t>
         </is>
       </c>
     </row>
@@ -22426,17 +22426,17 @@
       </c>
       <c r="K30" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:03</t>
+          <t xml:space="preserve">2:20</t>
         </is>
       </c>
       <c r="L30" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:21</t>
+          <t xml:space="preserve">2:39</t>
         </is>
       </c>
       <c r="M30" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:26</t>
+          <t xml:space="preserve">2:42</t>
         </is>
       </c>
     </row>
@@ -22485,17 +22485,17 @@
       </c>
       <c r="K31" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:03</t>
+          <t xml:space="preserve">2:20</t>
         </is>
       </c>
       <c r="L31" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:20</t>
+          <t xml:space="preserve">2:38</t>
         </is>
       </c>
       <c r="M31" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:26</t>
+          <t xml:space="preserve">2:42</t>
         </is>
       </c>
     </row>
@@ -22544,17 +22544,17 @@
       </c>
       <c r="K32" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:07</t>
+          <t xml:space="preserve">2:24</t>
         </is>
       </c>
       <c r="L32" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:20</t>
+          <t xml:space="preserve">2:38</t>
         </is>
       </c>
       <c r="M32" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:27</t>
+          <t xml:space="preserve">2:42</t>
         </is>
       </c>
     </row>
@@ -22603,17 +22603,17 @@
       </c>
       <c r="K33" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:09</t>
+          <t xml:space="preserve">1:18</t>
         </is>
       </c>
       <c r="L33" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:29</t>
+          <t xml:space="preserve">1:40</t>
         </is>
       </c>
       <c r="M33" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:27</t>
+          <t xml:space="preserve">2:42</t>
         </is>
       </c>
     </row>
@@ -22662,17 +22662,17 @@
       </c>
       <c r="K34" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:18</t>
+          <t xml:space="preserve">1:30</t>
         </is>
       </c>
       <c r="L34" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:39</t>
+          <t xml:space="preserve">1:52</t>
         </is>
       </c>
       <c r="M34" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:27</t>
+          <t xml:space="preserve">2:42</t>
         </is>
       </c>
     </row>
@@ -22721,17 +22721,17 @@
       </c>
       <c r="K35" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:21</t>
+          <t xml:space="preserve">1:33</t>
         </is>
       </c>
       <c r="L35" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:40</t>
+          <t xml:space="preserve">1:53</t>
         </is>
       </c>
       <c r="M35" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:27</t>
+          <t xml:space="preserve">2:43</t>
         </is>
       </c>
     </row>
@@ -22780,17 +22780,17 @@
       </c>
       <c r="K36" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:13</t>
+          <t xml:space="preserve">2:31</t>
         </is>
       </c>
       <c r="L36" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:29</t>
+          <t xml:space="preserve">2:49</t>
         </is>
       </c>
       <c r="M36" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:41</t>
+          <t xml:space="preserve">3:00</t>
         </is>
       </c>
     </row>
@@ -22839,17 +22839,17 @@
       </c>
       <c r="K37" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:14</t>
+          <t xml:space="preserve">2:31</t>
         </is>
       </c>
       <c r="L37" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:29</t>
+          <t xml:space="preserve">2:49</t>
         </is>
       </c>
       <c r="M37" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:41</t>
+          <t xml:space="preserve">3:00</t>
         </is>
       </c>
     </row>
@@ -22898,17 +22898,17 @@
       </c>
       <c r="K38" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:23</t>
+          <t xml:space="preserve">2:43</t>
         </is>
       </c>
       <c r="L38" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:39</t>
+          <t xml:space="preserve">3:00</t>
         </is>
       </c>
       <c r="M38" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:41</t>
+          <t xml:space="preserve">3:00</t>
         </is>
       </c>
     </row>
@@ -22957,17 +22957,17 @@
       </c>
       <c r="K39" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:47</t>
+          <t xml:space="preserve">0:53</t>
         </is>
       </c>
       <c r="L39" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:08</t>
+          <t xml:space="preserve">1:16</t>
         </is>
       </c>
       <c r="M39" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:41</t>
+          <t xml:space="preserve">3:00</t>
         </is>
       </c>
     </row>
@@ -23016,17 +23016,17 @@
       </c>
       <c r="K40" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:45</t>
+          <t xml:space="preserve">0:52</t>
         </is>
       </c>
       <c r="L40" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:09</t>
+          <t xml:space="preserve">1:17</t>
         </is>
       </c>
       <c r="M40" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:42</t>
+          <t xml:space="preserve">3:00</t>
         </is>
       </c>
     </row>
@@ -23075,17 +23075,17 @@
       </c>
       <c r="K41" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:47</t>
+          <t xml:space="preserve">0:54</t>
         </is>
       </c>
       <c r="L41" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:08</t>
+          <t xml:space="preserve">1:16</t>
         </is>
       </c>
       <c r="M41" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:42</t>
+          <t xml:space="preserve">3:00</t>
         </is>
       </c>
     </row>
@@ -23134,17 +23134,17 @@
       </c>
       <c r="K42" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:17</t>
+          <t xml:space="preserve">2:35</t>
         </is>
       </c>
       <c r="L42" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:30</t>
+          <t xml:space="preserve">2:50</t>
         </is>
       </c>
       <c r="M42" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:56</t>
+          <t xml:space="preserve">3:15</t>
         </is>
       </c>
     </row>
@@ -23193,17 +23193,17 @@
       </c>
       <c r="K43" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:23</t>
+          <t xml:space="preserve">2:43</t>
         </is>
       </c>
       <c r="L43" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:40</t>
+          <t xml:space="preserve">3:01</t>
         </is>
       </c>
       <c r="M43" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:56</t>
+          <t xml:space="preserve">3:15</t>
         </is>
       </c>
     </row>
@@ -23252,17 +23252,17 @@
       </c>
       <c r="K44" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:28</t>
+          <t xml:space="preserve">2:48</t>
         </is>
       </c>
       <c r="L44" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:41</t>
+          <t xml:space="preserve">3:03</t>
         </is>
       </c>
       <c r="M44" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:57</t>
+          <t xml:space="preserve">3:15</t>
         </is>
       </c>
     </row>
@@ -23311,17 +23311,17 @@
       </c>
       <c r="K45" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:57</t>
+          <t xml:space="preserve">1:05</t>
         </is>
       </c>
       <c r="L45" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:21</t>
+          <t xml:space="preserve">1:31</t>
         </is>
       </c>
       <c r="M45" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:57</t>
+          <t xml:space="preserve">3:15</t>
         </is>
       </c>
     </row>
@@ -23370,17 +23370,17 @@
       </c>
       <c r="K46" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:55</t>
+          <t xml:space="preserve">1:03</t>
         </is>
       </c>
       <c r="L46" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:19</t>
+          <t xml:space="preserve">1:29</t>
         </is>
       </c>
       <c r="M46" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:57</t>
+          <t xml:space="preserve">3:16</t>
         </is>
       </c>
     </row>
@@ -23429,17 +23429,17 @@
       </c>
       <c r="K47" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:57</t>
+          <t xml:space="preserve">1:05</t>
         </is>
       </c>
       <c r="L47" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:19</t>
+          <t xml:space="preserve">1:29</t>
         </is>
       </c>
       <c r="M47" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:57</t>
+          <t xml:space="preserve">3:16</t>
         </is>
       </c>
     </row>
@@ -23488,17 +23488,17 @@
       </c>
       <c r="K48" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:39</t>
+          <t xml:space="preserve">3:00</t>
         </is>
       </c>
       <c r="L48" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:51</t>
+          <t xml:space="preserve">3:14</t>
         </is>
       </c>
       <c r="M48" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:13</t>
+          <t xml:space="preserve">3:39</t>
         </is>
       </c>
     </row>
@@ -23547,17 +23547,17 @@
       </c>
       <c r="K49" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:50</t>
+          <t xml:space="preserve">3:13</t>
         </is>
       </c>
       <c r="L49" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:00</t>
+          <t xml:space="preserve">3:26</t>
         </is>
       </c>
       <c r="M49" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:14</t>
+          <t xml:space="preserve">3:39</t>
         </is>
       </c>
     </row>
@@ -23606,17 +23606,17 @@
       </c>
       <c r="K50" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:00</t>
+          <t xml:space="preserve">3:26</t>
         </is>
       </c>
       <c r="L50" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:11</t>
+          <t xml:space="preserve">3:38</t>
         </is>
       </c>
       <c r="M50" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:14</t>
+          <t xml:space="preserve">3:40</t>
         </is>
       </c>
     </row>
@@ -23665,17 +23665,17 @@
       </c>
       <c r="K51" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:24</t>
+          <t xml:space="preserve">0:27</t>
         </is>
       </c>
       <c r="L51" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:48</t>
+          <t xml:space="preserve">0:53</t>
         </is>
       </c>
       <c r="M51" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:14</t>
+          <t xml:space="preserve">3:40</t>
         </is>
       </c>
     </row>
@@ -23724,17 +23724,17 @@
       </c>
       <c r="K52" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:22</t>
+          <t xml:space="preserve">0:25</t>
         </is>
       </c>
       <c r="L52" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:48</t>
+          <t xml:space="preserve">0:53</t>
         </is>
       </c>
       <c r="M52" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:14</t>
+          <t xml:space="preserve">3:40</t>
         </is>
       </c>
     </row>
@@ -23783,17 +23783,17 @@
       </c>
       <c r="K53" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:25</t>
+          <t xml:space="preserve">0:28</t>
         </is>
       </c>
       <c r="L53" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:48</t>
+          <t xml:space="preserve">0:53</t>
         </is>
       </c>
       <c r="M53" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:14</t>
+          <t xml:space="preserve">3:40</t>
         </is>
       </c>
     </row>
@@ -23842,17 +23842,17 @@
       </c>
       <c r="K54" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:11</t>
+          <t xml:space="preserve">3:38</t>
         </is>
       </c>
       <c r="L54" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:22</t>
+          <t xml:space="preserve">3:51</t>
         </is>
       </c>
       <c r="M54" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:46</t>
+          <t xml:space="preserve">4:17</t>
         </is>
       </c>
     </row>
@@ -23901,17 +23901,17 @@
       </c>
       <c r="K55" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:21</t>
+          <t xml:space="preserve">3:50</t>
         </is>
       </c>
       <c r="L55" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:33</t>
+          <t xml:space="preserve">4:03</t>
         </is>
       </c>
       <c r="M55" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:46</t>
+          <t xml:space="preserve">4:17</t>
         </is>
       </c>
     </row>
@@ -23960,17 +23960,17 @@
       </c>
       <c r="K56" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:32</t>
+          <t xml:space="preserve">4:02</t>
         </is>
       </c>
       <c r="L56" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:44</t>
+          <t xml:space="preserve">4:16</t>
         </is>
       </c>
       <c r="M56" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:46</t>
+          <t xml:space="preserve">4:17</t>
         </is>
       </c>
     </row>
@@ -24019,17 +24019,17 @@
       </c>
       <c r="K57" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:35</t>
+          <t xml:space="preserve">0:40</t>
         </is>
       </c>
       <c r="L57" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:59</t>
+          <t xml:space="preserve">1:06</t>
         </is>
       </c>
       <c r="M57" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:47</t>
+          <t xml:space="preserve">4:17</t>
         </is>
       </c>
     </row>
@@ -24078,17 +24078,17 @@
       </c>
       <c r="K58" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:35</t>
+          <t xml:space="preserve">0:39</t>
         </is>
       </c>
       <c r="L58" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:59</t>
+          <t xml:space="preserve">1:05</t>
         </is>
       </c>
       <c r="M58" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:47</t>
+          <t xml:space="preserve">4:17</t>
         </is>
       </c>
     </row>
@@ -24137,17 +24137,17 @@
       </c>
       <c r="K59" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:33</t>
+          <t xml:space="preserve">0:38</t>
         </is>
       </c>
       <c r="L59" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:58</t>
+          <t xml:space="preserve">1:05</t>
         </is>
       </c>
       <c r="M59" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:47</t>
+          <t xml:space="preserve">4:17</t>
         </is>
       </c>
     </row>
@@ -24196,17 +24196,17 @@
       </c>
       <c r="K60" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:35</t>
+          <t xml:space="preserve">2:56</t>
         </is>
       </c>
       <c r="L60" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:48</t>
+          <t xml:space="preserve">3:10</t>
         </is>
       </c>
       <c r="M60" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:02</t>
+          <t xml:space="preserve">4:33</t>
         </is>
       </c>
     </row>
@@ -24255,17 +24255,17 @@
       </c>
       <c r="K61" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:35</t>
+          <t xml:space="preserve">2:56</t>
         </is>
       </c>
       <c r="L61" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:47</t>
+          <t xml:space="preserve">3:09</t>
         </is>
       </c>
       <c r="M61" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:02</t>
+          <t xml:space="preserve">4:33</t>
         </is>
       </c>
     </row>
@@ -24314,17 +24314,17 @@
       </c>
       <c r="K62" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:45</t>
+          <t xml:space="preserve">3:07</t>
         </is>
       </c>
       <c r="L62" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:57</t>
+          <t xml:space="preserve">3:20</t>
         </is>
       </c>
       <c r="M62" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:02</t>
+          <t xml:space="preserve">4:33</t>
         </is>
       </c>
     </row>
@@ -24378,12 +24378,12 @@
       </c>
       <c r="L63" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:31</t>
+          <t xml:space="preserve">0:32</t>
         </is>
       </c>
       <c r="M63" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:03</t>
+          <t xml:space="preserve">4:33</t>
         </is>
       </c>
     </row>
@@ -24432,17 +24432,17 @@
       </c>
       <c r="K64" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:15</t>
+          <t xml:space="preserve">0:16</t>
         </is>
       </c>
       <c r="L64" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:39</t>
+          <t xml:space="preserve">0:42</t>
         </is>
       </c>
       <c r="M64" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:03</t>
+          <t xml:space="preserve">4:33</t>
         </is>
       </c>
     </row>
@@ -24496,12 +24496,12 @@
       </c>
       <c r="L65" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:32</t>
+          <t xml:space="preserve">0:33</t>
         </is>
       </c>
       <c r="M65" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:03</t>
+          <t xml:space="preserve">4:33</t>
         </is>
       </c>
     </row>
@@ -24550,17 +24550,17 @@
       </c>
       <c r="K66" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">2:54</t>
+          <t xml:space="preserve">3:17</t>
         </is>
       </c>
       <c r="L66" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:05</t>
+          <t xml:space="preserve">3:29</t>
         </is>
       </c>
       <c r="M66" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:16</t>
+          <t xml:space="preserve">4:47</t>
         </is>
       </c>
     </row>
@@ -24609,17 +24609,17 @@
       </c>
       <c r="K67" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:02</t>
+          <t xml:space="preserve">3:26</t>
         </is>
       </c>
       <c r="L67" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:12</t>
+          <t xml:space="preserve">3:38</t>
         </is>
       </c>
       <c r="M67" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:16</t>
+          <t xml:space="preserve">4:47</t>
         </is>
       </c>
     </row>
@@ -24668,17 +24668,17 @@
       </c>
       <c r="K68" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:09</t>
+          <t xml:space="preserve">3:35</t>
         </is>
       </c>
       <c r="L68" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">3:19</t>
+          <t xml:space="preserve">3:46</t>
         </is>
       </c>
       <c r="M68" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:17</t>
+          <t xml:space="preserve">4:47</t>
         </is>
       </c>
     </row>
@@ -24727,17 +24727,17 @@
       </c>
       <c r="K69" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:14</t>
+          <t xml:space="preserve">0:15</t>
         </is>
       </c>
       <c r="L69" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:39</t>
+          <t xml:space="preserve">0:41</t>
         </is>
       </c>
       <c r="M69" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:17</t>
+          <t xml:space="preserve">4:47</t>
         </is>
       </c>
     </row>
@@ -24796,7 +24796,7 @@
       </c>
       <c r="M70" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:17</t>
+          <t xml:space="preserve">4:47</t>
         </is>
       </c>
     </row>
@@ -24845,17 +24845,17 @@
       </c>
       <c r="K71" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:13</t>
+          <t xml:space="preserve">0:14</t>
         </is>
       </c>
       <c r="L71" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">0:35</t>
+          <t xml:space="preserve">0:37</t>
         </is>
       </c>
       <c r="M71" s="342" t="inlineStr">
         <is>
-          <t xml:space="preserve">4:17</t>
+          <t xml:space="preserve">4:47</t>
         </is>
       </c>
     </row>

</xml_diff>